<commit_message>
Break glass new as global admin
</commit_message>
<xml_diff>
--- a/data/aad/Rollen.xlsx
+++ b/data/aad/Rollen.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CCC5043-0B0C-484D-AAFD-FEE950D838AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E48F51C2-ECE3-43FC-B049-D4F3EFF7718E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2652" yWindow="2652" windowWidth="30960" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3972" yWindow="2340" windowWidth="30960" windowHeight="12168" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="setupRoles" sheetId="1" r:id="rId1"/>
@@ -803,6 +803,9 @@
       <c r="A2" s="4" t="s">
         <v>78</v>
       </c>
+      <c r="B2" t="s">
+        <v>87</v>
+      </c>
       <c r="C2" s="3" t="s">
         <v>88</v>
       </c>
@@ -813,9 +816,6 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>87</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>88</v>

</xml_diff>